<commit_message>
fin de la partie 2
</commit_message>
<xml_diff>
--- a/mesures/TP 2.xlsx
+++ b/mesures/TP 2.xlsx
@@ -12,6 +12,9 @@
     <sheet name="1.1 Geant4" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="1.2 BERT" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Synthèse" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="2 Questions" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="2 Quantiles" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="2 EcoIndex" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="175">
   <si>
     <t xml:space="preserve">TP 2 – Constantes (Lannelongue et al., 2021)</t>
   </si>
@@ -416,13 +419,164 @@
   </si>
   <si>
     <t xml:space="preserve">Valeurs « Article » : Lannelongue et al., Adv. Sci. 2021, 8, 2100707, §2.1 et §2.3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partie 2 – EcoIndex : réponses aux questions 1 à 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1 – Formule implémentée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EcoIndex = 100 − 5 × (3 × Q_dom + 2 × Q_req + Q_size) / 6
+Pondérations : 3 pour la taille du DOM, 2 pour le nombre de requêtes, 1 pour le poids de la page. Le score va de 0 à 100 (100 = meilleur).
+Vérifié dans le code de l'organisation GitHub cnumr :
+• cnumr/ecoindex_python, components/ecoindex/compute/ecoindex.py, get_score() : round(100 - 5 * (3 * q_dom + 2 * q_req + q_size) / 6)
+• cnumr/ecoindex_js, src/index.js, computeEcoIndex() : même formule, sans arrondi.
+Les deux implémentations lisent les mêmes bornes (cnumr/ecoindex_reference) : les quantiles copiés dans ecoindex_python sont identiques au fichier de référence.
+Le code calcule aussi la note (A ≥ 80 &lt; B … G), les GES = 2 + 2 × (50 − EcoIndex) / 100 (gCO2e) et l'eau = 3 + 3 × (50 − EcoIndex) / 100 (cl).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2 – Fonction Quantile(x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour un tableau de bornes Q[0..20] (21 bornes, 20 intervalles) et une valeur x :
+• on cherche le premier i (de 1 à 20) tel que x &lt; Q[i] ;
+• Quantile(x) = (i − 1) + (x − Q[i−1]) / (Q[i] − Q[i−1])   (interpolation linéaire dans l'intervalle) ;
+• si x ≥ Q[20], Quantile(x) = 20.
+Le résultat est donc un réel entre 0 et 20 : 0 = meilleur que toutes les pages de référence, 20 = pire.
+Dans la feuille « 2 EcoIndex », il est implémenté avec EQUIV (MATCH) et INDEX sur l'onglet « 2 Quantiles ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3 – Scénario d'évaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scénario du scraper officiel (ecoindex_python, scraper/scrap.py) :
+1. Navigateur de bureau sans tête, contexte neuf (cache vide, sans cookies de consentement), user-agent desktop.
+2. Fenêtre 1920 × 1080 px.
+3. Chargement de l'URL et attente de l'événement load.
+4. Attente avant défilement (1 s par défaut, 3 s via le helper), capture d'écran.
+5. Touche Flèche bas puis défilement jusqu'en bas de page (déclenche le lazy-loading).
+6. Attente après défilement (1 à 3 s).
+7. Mesures : DOM = nombre d'éléments (*) hors enfants des &lt;svg&gt; ; requêtes = nombre d'entrées du fichier HAR ; poids = somme des tailles transférées / 1000 (Ko).
+On mesure la page d'accueil, telle qu'un visiteur la découvre, sans accepter les cookies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4 – Bornes de quantiles (cnumr/ecoindex_reference, ecoindex_reference.json)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOM (éléments)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requêtes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poids (Ko)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seuils de notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note = première lettre dont le score est strictement supérieur au seuil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q5 – Calcul de l'EcoIndex des pages d'accueil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrées (bleu, jaune) : mesures DOM / requêtes / poids relevées par ecoindex.fr (API publique bff.ecoindex.fr). Tout le reste est calculé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q_dom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q_req</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q_size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EcoIndex (non arrondi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EcoIndex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GES (gCO2e)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eau (cl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ecoindex.fr : score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date et remarque de la mesure ecoindex.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ecoindex.fr/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.leboncoin.fr/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19/03/2026 – mesures plus récentes écartées : 48 éléments / 9 requêtes = page anti-robot d'Amazon, pas la vraie page d'accueil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérification : un écart de 0 en colonne O signifie que la feuille retrouve exactement le score d'ecoindex.fr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les mesures d'un même site varient d'un passage à l'autre (publicités, contenus dynamiques) : on retient la mesure la plus récente qui reflète la vraie page.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
@@ -436,6 +590,7 @@
     <numFmt numFmtId="174" formatCode="#,##0.0"/>
     <numFmt numFmtId="175" formatCode="#,##0;\-#,##0;\-"/>
     <numFmt numFmtId="176" formatCode="0.00%"/>
+    <numFmt numFmtId="177" formatCode="0;\-0;0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -593,7 +748,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -720,6 +875,54 @@
     </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2033,4 +2236,724 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="32" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>137</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="29" t="n">
+        <v>47</v>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="34" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="n">
+        <v>75</v>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>15</v>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>159</v>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>319.53</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>233</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>34</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>479.46</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>298</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>42</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>631.97</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>358</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>49</v>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>783.38</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>417</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>56</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>937.91</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>63</v>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>1098.62</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="29" t="n">
+        <v>537</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>70</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>1265.47</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>603</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>78</v>
+      </c>
+      <c r="D14" s="34" t="n">
+        <v>1448.32</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>674</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>86</v>
+      </c>
+      <c r="D15" s="34" t="n">
+        <v>1648.27</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="29" t="n">
+        <v>753</v>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>95</v>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>1876.08</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="29" t="n">
+        <v>843</v>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>105</v>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>2142.06</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>949</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>117</v>
+      </c>
+      <c r="D18" s="34" t="n">
+        <v>2465.37</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>1076</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>130</v>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>2866.31</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="29" t="n">
+        <v>1237</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>147</v>
+      </c>
+      <c r="D20" s="34" t="n">
+        <v>3401.59</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>1459</v>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>170</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>4155.73</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>1801</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>205</v>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>5400.08</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="29" t="n">
+        <v>2479</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>281</v>
+      </c>
+      <c r="D23" s="34" t="n">
+        <v>8037.54</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="29" t="n">
+        <v>594601</v>
+      </c>
+      <c r="C24" s="29" t="n">
+        <v>3920</v>
+      </c>
+      <c r="D24" s="34" t="n">
+        <v>223212.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="G4" s="36" t="s">
+        <v>157</v>
+      </c>
+      <c r="H4" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="J4" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="K4" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="L4" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="M4" s="36" t="s">
+        <v>163</v>
+      </c>
+      <c r="N4" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="O4" s="36" t="s">
+        <v>165</v>
+      </c>
+      <c r="P4" s="36" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="37" t="n">
+        <v>155.329</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <f aca="false">IF(B5&gt;=MAX('2 Quantiles'!$B$4:$B$24),20,MATCH(B5,'2 Quantiles'!$B$4:$B$24,1)-1+(B5-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B5,'2 Quantiles'!$B$4:$B$24,1)))/(INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B5,'2 Quantiles'!$B$4:$B$24,1)+1)-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B5,'2 Quantiles'!$B$4:$B$24,1))))</f>
+        <v>3.48648648648649</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <f aca="false">IF(C5&gt;=MAX('2 Quantiles'!$C$4:$C$24),20,MATCH(C5,'2 Quantiles'!$C$4:$C$24,1)-1+(C5-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C5,'2 Quantiles'!$C$4:$C$24,1)))/(INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C5,'2 Quantiles'!$C$4:$C$24,1)+1)-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C5,'2 Quantiles'!$C$4:$C$24,1))))</f>
+        <v>1.23076923076923</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <f aca="false">IF(D5&gt;=MAX('2 Quantiles'!$D$4:$D$24),20,MATCH(D5,'2 Quantiles'!$D$4:$D$24,1)-1+(D5-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D5,'2 Quantiles'!$D$4:$D$24,1)))/(INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D5,'2 Quantiles'!$D$4:$D$24,1)+1)-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D5,'2 Quantiles'!$D$4:$D$24,1))))</f>
+        <v>2.06079620202482</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <f aca="false">100-5*(3*E5+2*F5+G5)/6</f>
+        <v>87.5151715641477</v>
+      </c>
+      <c r="I5" s="38" t="n">
+        <f aca="false">ROUND(H5,0)</f>
+        <v>88</v>
+      </c>
+      <c r="J5" s="39" t="str">
+        <f aca="false">IF(I5&gt;'2 Quantiles'!$G$4,"A",IF(I5&gt;'2 Quantiles'!$G$5,"B",IF(I5&gt;'2 Quantiles'!$G$6,"C",IF(I5&gt;'2 Quantiles'!$G$7,"D",IF(I5&gt;'2 Quantiles'!$G$8,"E",IF(I5&gt;'2 Quantiles'!$G$9,"F","G"))))))</f>
+        <v>A</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <f aca="false">ROUND(2+2*(50-I5)/100,2)</f>
+        <v>1.24</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <f aca="false">ROUND(3+3*(50-I5)/100,2)</f>
+        <v>1.86</v>
+      </c>
+      <c r="M5" s="40" t="n">
+        <v>88</v>
+      </c>
+      <c r="N5" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="O5" s="42" t="n">
+        <f aca="false">I5-M5</f>
+        <v>0</v>
+      </c>
+      <c r="P5" s="43" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1462</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>176</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>4374.26</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <f aca="false">IF(B6&gt;=MAX('2 Quantiles'!$B$4:$B$24),20,MATCH(B6,'2 Quantiles'!$B$4:$B$24,1)-1+(B6-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B6,'2 Quantiles'!$B$4:$B$24,1)))/(INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B6,'2 Quantiles'!$B$4:$B$24,1)+1)-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B6,'2 Quantiles'!$B$4:$B$24,1))))</f>
+        <v>17.0087719298246</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <f aca="false">IF(C6&gt;=MAX('2 Quantiles'!$C$4:$C$24),20,MATCH(C6,'2 Quantiles'!$C$4:$C$24,1)-1+(C6-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C6,'2 Quantiles'!$C$4:$C$24,1)))/(INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C6,'2 Quantiles'!$C$4:$C$24,1)+1)-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C6,'2 Quantiles'!$C$4:$C$24,1))))</f>
+        <v>17.1714285714286</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <f aca="false">IF(D6&gt;=MAX('2 Quantiles'!$D$4:$D$24),20,MATCH(D6,'2 Quantiles'!$D$4:$D$24,1)-1+(D6-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D6,'2 Quantiles'!$D$4:$D$24,1)))/(INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D6,'2 Quantiles'!$D$4:$D$24,1)+1)-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D6,'2 Quantiles'!$D$4:$D$24,1))))</f>
+        <v>17.1756177924217</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">100-5*(3*E6+2*F6+G6)/6</f>
+        <v>14.5460077293728</v>
+      </c>
+      <c r="I6" s="38" t="n">
+        <f aca="false">ROUND(H6,0)</f>
+        <v>15</v>
+      </c>
+      <c r="J6" s="39" t="str">
+        <f aca="false">IF(I6&gt;'2 Quantiles'!$G$4,"A",IF(I6&gt;'2 Quantiles'!$G$5,"B",IF(I6&gt;'2 Quantiles'!$G$6,"C",IF(I6&gt;'2 Quantiles'!$G$7,"D",IF(I6&gt;'2 Quantiles'!$G$8,"E",IF(I6&gt;'2 Quantiles'!$G$9,"F","G"))))))</f>
+        <v>F</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <f aca="false">ROUND(2+2*(50-I6)/100,2)</f>
+        <v>2.7</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <f aca="false">ROUND(3+3*(50-I6)/100,2)</f>
+        <v>4.05</v>
+      </c>
+      <c r="M6" s="40" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="O6" s="42" t="n">
+        <f aca="false">I6-M6</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="43" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>2299</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>340</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>6019.26</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <f aca="false">IF(B7&gt;=MAX('2 Quantiles'!$B$4:$B$24),20,MATCH(B7,'2 Quantiles'!$B$4:$B$24,1)-1+(B7-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B7,'2 Quantiles'!$B$4:$B$24,1)))/(INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B7,'2 Quantiles'!$B$4:$B$24,1)+1)-INDEX('2 Quantiles'!$B$4:$B$24,MATCH(B7,'2 Quantiles'!$B$4:$B$24,1))))</f>
+        <v>18.7345132743363</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <f aca="false">IF(C7&gt;=MAX('2 Quantiles'!$C$4:$C$24),20,MATCH(C7,'2 Quantiles'!$C$4:$C$24,1)-1+(C7-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C7,'2 Quantiles'!$C$4:$C$24,1)))/(INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C7,'2 Quantiles'!$C$4:$C$24,1)+1)-INDEX('2 Quantiles'!$C$4:$C$24,MATCH(C7,'2 Quantiles'!$C$4:$C$24,1))))</f>
+        <v>19.0162132453971</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <f aca="false">IF(D7&gt;=MAX('2 Quantiles'!$D$4:$D$24),20,MATCH(D7,'2 Quantiles'!$D$4:$D$24,1)-1+(D7-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D7,'2 Quantiles'!$D$4:$D$24,1)))/(INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D7,'2 Quantiles'!$D$4:$D$24,1)+1)-INDEX('2 Quantiles'!$D$4:$D$24,MATCH(D7,'2 Quantiles'!$D$4:$D$24,1))))</f>
+        <v>18.2347637499716</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <f aca="false">100-5*(3*E7+2*F7+G7)/6</f>
+        <v>6.27439161352118</v>
+      </c>
+      <c r="I7" s="38" t="n">
+        <f aca="false">ROUND(H7,0)</f>
+        <v>6</v>
+      </c>
+      <c r="J7" s="39" t="str">
+        <f aca="false">IF(I7&gt;'2 Quantiles'!$G$4,"A",IF(I7&gt;'2 Quantiles'!$G$5,"B",IF(I7&gt;'2 Quantiles'!$G$6,"C",IF(I7&gt;'2 Quantiles'!$G$7,"D",IF(I7&gt;'2 Quantiles'!$G$8,"E",IF(I7&gt;'2 Quantiles'!$G$9,"F","G"))))))</f>
+        <v>G</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <f aca="false">ROUND(2+2*(50-I7)/100,2)</f>
+        <v>2.88</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <f aca="false">ROUND(3+3*(50-I7)/100,2)</f>
+        <v>4.32</v>
+      </c>
+      <c r="M7" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="O7" s="42" t="n">
+        <f aca="false">I7-M7</f>
+        <v>0</v>
+      </c>
+      <c r="P7" s="43" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>